<commit_message>
Variables de metadatos panel de hogares
</commit_message>
<xml_diff>
--- a/data-raw/xlsx/tabla_etiquetas.xlsx
+++ b/data-raw/xlsx/tabla_etiquetas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fernando_gallegos\Proyectos\odsa.eusilc\data-raw\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4517D1AB-8FB8-4F8F-8BC3-487FD50F3B8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFA112ED-33CC-4E64-B824-B633F54BD296}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11760" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$F$349</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$F$352</definedName>
   </definedNames>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1585" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1597" uniqueCount="466">
   <si>
     <t>variable</t>
   </si>
@@ -1417,6 +1417,15 @@
   </si>
   <si>
     <t>Cantidad de años presentes del grupo de rotación</t>
+  </si>
+  <si>
+    <t>hi08a</t>
+  </si>
+  <si>
+    <t>hi08b</t>
+  </si>
+  <si>
+    <t>hi08c</t>
   </si>
 </sst>
 </file>
@@ -1656,7 +1665,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F349"/>
+  <dimension ref="A1:F352"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" customWidth="1"/>
@@ -6280,63 +6289,63 @@
     </row>
     <row r="250" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
-        <v>291</v>
+        <v>463</v>
       </c>
       <c r="B250" t="s">
         <v>285</v>
       </c>
       <c r="C250" t="s">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="D250" t="s">
-        <v>292</v>
+        <v>35</v>
       </c>
     </row>
     <row r="251" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
-        <v>186</v>
+        <v>464</v>
       </c>
       <c r="B251" t="s">
         <v>285</v>
       </c>
       <c r="C251" t="s">
-        <v>187</v>
+        <v>8</v>
       </c>
       <c r="D251" t="s">
-        <v>293</v>
+        <v>37</v>
       </c>
     </row>
     <row r="252" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
-        <v>191</v>
+        <v>465</v>
       </c>
       <c r="B252" t="s">
         <v>285</v>
       </c>
       <c r="C252" t="s">
-        <v>187</v>
+        <v>8</v>
       </c>
       <c r="D252" t="s">
-        <v>294</v>
+        <v>462</v>
       </c>
     </row>
     <row r="253" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
-        <v>193</v>
+        <v>291</v>
       </c>
       <c r="B253" t="s">
         <v>285</v>
       </c>
       <c r="C253" t="s">
-        <v>187</v>
+        <v>39</v>
       </c>
       <c r="D253" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="254" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="B254" t="s">
         <v>285</v>
@@ -6345,12 +6354,12 @@
         <v>187</v>
       </c>
       <c r="D254" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
     </row>
     <row r="255" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="B255" t="s">
         <v>285</v>
@@ -6359,12 +6368,12 @@
         <v>187</v>
       </c>
       <c r="D255" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
     </row>
     <row r="256" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B256" t="s">
         <v>285</v>
@@ -6373,12 +6382,12 @@
         <v>187</v>
       </c>
       <c r="D256" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
     </row>
     <row r="257" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="B257" t="s">
         <v>285</v>
@@ -6387,12 +6396,12 @@
         <v>187</v>
       </c>
       <c r="D257" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="B258" t="s">
         <v>285</v>
@@ -6401,12 +6410,12 @@
         <v>187</v>
       </c>
       <c r="D258" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
     </row>
     <row r="259" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="B259" t="s">
         <v>285</v>
@@ -6415,12 +6424,12 @@
         <v>187</v>
       </c>
       <c r="D259" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B260" t="s">
         <v>285</v>
@@ -6429,12 +6438,12 @@
         <v>187</v>
       </c>
       <c r="D260" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
     </row>
     <row r="261" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B261" t="s">
         <v>285</v>
@@ -6443,12 +6452,12 @@
         <v>187</v>
       </c>
       <c r="D261" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="262" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="B262" t="s">
         <v>285</v>
@@ -6457,12 +6466,12 @@
         <v>187</v>
       </c>
       <c r="D262" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
-        <v>189</v>
+        <v>207</v>
       </c>
       <c r="B263" t="s">
         <v>285</v>
@@ -6471,12 +6480,12 @@
         <v>187</v>
       </c>
       <c r="D263" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
     </row>
     <row r="264" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
-        <v>306</v>
+        <v>209</v>
       </c>
       <c r="B264" t="s">
         <v>285</v>
@@ -6485,12 +6494,12 @@
         <v>187</v>
       </c>
       <c r="D264" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
     </row>
     <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
-        <v>308</v>
+        <v>211</v>
       </c>
       <c r="B265" t="s">
         <v>285</v>
@@ -6499,12 +6508,12 @@
         <v>187</v>
       </c>
       <c r="D265" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
     </row>
     <row r="266" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
-        <v>310</v>
+        <v>189</v>
       </c>
       <c r="B266" t="s">
         <v>285</v>
@@ -6513,12 +6522,12 @@
         <v>187</v>
       </c>
       <c r="D266" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
       <c r="B267" t="s">
         <v>285</v>
@@ -6527,12 +6536,12 @@
         <v>187</v>
       </c>
       <c r="D267" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
     </row>
     <row r="268" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="B268" t="s">
         <v>285</v>
@@ -6541,12 +6550,12 @@
         <v>187</v>
       </c>
       <c r="D268" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="B269" t="s">
         <v>285</v>
@@ -6555,12 +6564,12 @@
         <v>187</v>
       </c>
       <c r="D269" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="B270" t="s">
         <v>285</v>
@@ -6569,12 +6578,12 @@
         <v>187</v>
       </c>
       <c r="D270" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="B271" t="s">
         <v>285</v>
@@ -6583,12 +6592,12 @@
         <v>187</v>
       </c>
       <c r="D271" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
     </row>
     <row r="272" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="B272" t="s">
         <v>285</v>
@@ -6597,12 +6606,12 @@
         <v>187</v>
       </c>
       <c r="D272" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
     </row>
     <row r="273" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="B273" t="s">
         <v>285</v>
@@ -6611,12 +6620,12 @@
         <v>187</v>
       </c>
       <c r="D273" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
     </row>
     <row r="274" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="B274" t="s">
         <v>285</v>
@@ -6625,12 +6634,12 @@
         <v>187</v>
       </c>
       <c r="D274" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="B275" t="s">
         <v>285</v>
@@ -6639,12 +6648,12 @@
         <v>187</v>
       </c>
       <c r="D275" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="B276" t="s">
         <v>285</v>
@@ -6653,12 +6662,12 @@
         <v>187</v>
       </c>
       <c r="D276" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="B277" t="s">
         <v>285</v>
@@ -6667,12 +6676,12 @@
         <v>187</v>
       </c>
       <c r="D277" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
     </row>
     <row r="278" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
       <c r="B278" t="s">
         <v>285</v>
@@ -6681,12 +6690,12 @@
         <v>187</v>
       </c>
       <c r="D278" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
     </row>
     <row r="279" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="B279" t="s">
         <v>285</v>
@@ -6695,12 +6704,12 @@
         <v>187</v>
       </c>
       <c r="D279" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
     </row>
     <row r="280" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="B280" t="s">
         <v>285</v>
@@ -6709,12 +6718,12 @@
         <v>187</v>
       </c>
       <c r="D280" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A281" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
       <c r="B281" t="s">
         <v>285</v>
@@ -6723,12 +6732,12 @@
         <v>187</v>
       </c>
       <c r="D281" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
     </row>
     <row r="282" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A282" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="B282" t="s">
         <v>285</v>
@@ -6737,12 +6746,12 @@
         <v>187</v>
       </c>
       <c r="D282" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
     </row>
     <row r="283" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
       <c r="B283" t="s">
         <v>285</v>
@@ -6751,12 +6760,12 @@
         <v>187</v>
       </c>
       <c r="D283" t="s">
-        <v>345</v>
+        <v>339</v>
       </c>
     </row>
     <row r="284" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A284" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="B284" t="s">
         <v>285</v>
@@ -6765,12 +6774,12 @@
         <v>187</v>
       </c>
       <c r="D284" t="s">
-        <v>347</v>
+        <v>341</v>
       </c>
     </row>
     <row r="285" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A285" t="s">
-        <v>348</v>
+        <v>342</v>
       </c>
       <c r="B285" t="s">
         <v>285</v>
@@ -6779,12 +6788,12 @@
         <v>187</v>
       </c>
       <c r="D285" t="s">
-        <v>349</v>
+        <v>343</v>
       </c>
     </row>
     <row r="286" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
-        <v>350</v>
+        <v>344</v>
       </c>
       <c r="B286" t="s">
         <v>285</v>
@@ -6793,12 +6802,12 @@
         <v>187</v>
       </c>
       <c r="D286" t="s">
-        <v>351</v>
+        <v>345</v>
       </c>
     </row>
     <row r="287" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
-        <v>352</v>
+        <v>346</v>
       </c>
       <c r="B287" t="s">
         <v>285</v>
@@ -6807,12 +6816,12 @@
         <v>187</v>
       </c>
       <c r="D287" t="s">
-        <v>353</v>
+        <v>347</v>
       </c>
     </row>
     <row r="288" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A288" t="s">
-        <v>354</v>
+        <v>348</v>
       </c>
       <c r="B288" t="s">
         <v>285</v>
@@ -6821,12 +6830,12 @@
         <v>187</v>
       </c>
       <c r="D288" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
     </row>
     <row r="289" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A289" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="B289" t="s">
         <v>285</v>
@@ -6835,12 +6844,12 @@
         <v>187</v>
       </c>
       <c r="D289" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
     </row>
     <row r="290" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A290" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="B290" t="s">
         <v>285</v>
@@ -6849,12 +6858,12 @@
         <v>187</v>
       </c>
       <c r="D290" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
     </row>
     <row r="291" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A291" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="B291" t="s">
         <v>285</v>
@@ -6863,12 +6872,12 @@
         <v>187</v>
       </c>
       <c r="D291" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
     </row>
     <row r="292" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A292" t="s">
-        <v>362</v>
+        <v>356</v>
       </c>
       <c r="B292" t="s">
         <v>285</v>
@@ -6877,12 +6886,12 @@
         <v>187</v>
       </c>
       <c r="D292" t="s">
-        <v>363</v>
+        <v>357</v>
       </c>
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" t="s">
-        <v>217</v>
+        <v>358</v>
       </c>
       <c r="B293" t="s">
         <v>285</v>
@@ -6891,12 +6900,12 @@
         <v>187</v>
       </c>
       <c r="D293" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
     </row>
     <row r="294" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
-        <v>221</v>
+        <v>360</v>
       </c>
       <c r="B294" t="s">
         <v>285</v>
@@ -6905,12 +6914,12 @@
         <v>187</v>
       </c>
       <c r="D294" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
     </row>
     <row r="295" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
-        <v>223</v>
+        <v>362</v>
       </c>
       <c r="B295" t="s">
         <v>285</v>
@@ -6919,12 +6928,12 @@
         <v>187</v>
       </c>
       <c r="D295" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
     </row>
     <row r="296" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="B296" t="s">
         <v>285</v>
@@ -6933,12 +6942,12 @@
         <v>187</v>
       </c>
       <c r="D296" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
     </row>
     <row r="297" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="B297" t="s">
         <v>285</v>
@@ -6947,12 +6956,12 @@
         <v>187</v>
       </c>
       <c r="D297" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
     </row>
     <row r="298" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="B298" t="s">
         <v>285</v>
@@ -6961,12 +6970,12 @@
         <v>187</v>
       </c>
       <c r="D298" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="299" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B299" t="s">
         <v>285</v>
@@ -6975,12 +6984,12 @@
         <v>187</v>
       </c>
       <c r="D299" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A300" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="B300" t="s">
         <v>285</v>
@@ -6989,12 +6998,12 @@
         <v>187</v>
       </c>
       <c r="D300" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
     </row>
     <row r="301" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A301" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="B301" t="s">
         <v>285</v>
@@ -7003,12 +7012,12 @@
         <v>187</v>
       </c>
       <c r="D301" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
     </row>
     <row r="302" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A302" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="B302" t="s">
         <v>285</v>
@@ -7017,12 +7026,12 @@
         <v>187</v>
       </c>
       <c r="D302" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
     </row>
     <row r="303" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A303" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="B303" t="s">
         <v>285</v>
@@ -7031,12 +7040,12 @@
         <v>187</v>
       </c>
       <c r="D303" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="304" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A304" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="B304" t="s">
         <v>285</v>
@@ -7045,12 +7054,12 @@
         <v>187</v>
       </c>
       <c r="D304" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="305" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A305" t="s">
-        <v>219</v>
+        <v>237</v>
       </c>
       <c r="B305" t="s">
         <v>285</v>
@@ -7059,12 +7068,12 @@
         <v>187</v>
       </c>
       <c r="D305" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="306" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A306" t="s">
-        <v>377</v>
+        <v>239</v>
       </c>
       <c r="B306" t="s">
         <v>285</v>
@@ -7073,12 +7082,12 @@
         <v>187</v>
       </c>
       <c r="D306" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
     </row>
     <row r="307" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A307" t="s">
-        <v>379</v>
+        <v>241</v>
       </c>
       <c r="B307" t="s">
         <v>285</v>
@@ -7087,12 +7096,12 @@
         <v>187</v>
       </c>
       <c r="D307" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
     </row>
     <row r="308" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
-        <v>381</v>
+        <v>219</v>
       </c>
       <c r="B308" t="s">
         <v>285</v>
@@ -7101,12 +7110,12 @@
         <v>187</v>
       </c>
       <c r="D308" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
     </row>
     <row r="309" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A309" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="B309" t="s">
         <v>285</v>
@@ -7115,12 +7124,12 @@
         <v>187</v>
       </c>
       <c r="D309" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
     </row>
     <row r="310" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A310" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="B310" t="s">
         <v>285</v>
@@ -7129,12 +7138,12 @@
         <v>187</v>
       </c>
       <c r="D310" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
     </row>
     <row r="311" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A311" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="B311" t="s">
         <v>285</v>
@@ -7143,12 +7152,12 @@
         <v>187</v>
       </c>
       <c r="D311" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
     </row>
     <row r="312" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A312" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="B312" t="s">
         <v>285</v>
@@ -7157,12 +7166,12 @@
         <v>187</v>
       </c>
       <c r="D312" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A313" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
       <c r="B313" t="s">
         <v>285</v>
@@ -7171,12 +7180,12 @@
         <v>187</v>
       </c>
       <c r="D313" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
     </row>
     <row r="314" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A314" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="B314" t="s">
         <v>285</v>
@@ -7185,12 +7194,12 @@
         <v>187</v>
       </c>
       <c r="D314" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
     </row>
     <row r="315" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A315" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
       <c r="B315" t="s">
         <v>285</v>
@@ -7199,12 +7208,12 @@
         <v>187</v>
       </c>
       <c r="D315" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
     </row>
     <row r="316" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A316" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="B316" t="s">
         <v>285</v>
@@ -7213,12 +7222,12 @@
         <v>187</v>
       </c>
       <c r="D316" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
     </row>
     <row r="317" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A317" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="B317" t="s">
         <v>285</v>
@@ -7227,12 +7236,12 @@
         <v>187</v>
       </c>
       <c r="D317" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
     </row>
     <row r="318" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A318" t="s">
-        <v>401</v>
+        <v>395</v>
       </c>
       <c r="B318" t="s">
         <v>285</v>
@@ -7241,12 +7250,12 @@
         <v>187</v>
       </c>
       <c r="D318" t="s">
-        <v>402</v>
+        <v>396</v>
       </c>
     </row>
     <row r="319" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A319" t="s">
-        <v>403</v>
+        <v>397</v>
       </c>
       <c r="B319" t="s">
         <v>285</v>
@@ -7255,12 +7264,12 @@
         <v>187</v>
       </c>
       <c r="D319" t="s">
-        <v>404</v>
+        <v>398</v>
       </c>
     </row>
     <row r="320" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A320" t="s">
-        <v>405</v>
+        <v>399</v>
       </c>
       <c r="B320" t="s">
         <v>285</v>
@@ -7269,12 +7278,12 @@
         <v>187</v>
       </c>
       <c r="D320" t="s">
-        <v>406</v>
+        <v>400</v>
       </c>
     </row>
     <row r="321" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A321" t="s">
-        <v>407</v>
+        <v>401</v>
       </c>
       <c r="B321" t="s">
         <v>285</v>
@@ -7283,12 +7292,12 @@
         <v>187</v>
       </c>
       <c r="D321" t="s">
-        <v>408</v>
+        <v>402</v>
       </c>
     </row>
     <row r="322" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A322" t="s">
-        <v>409</v>
+        <v>403</v>
       </c>
       <c r="B322" t="s">
         <v>285</v>
@@ -7297,12 +7306,12 @@
         <v>187</v>
       </c>
       <c r="D322" t="s">
-        <v>410</v>
+        <v>404</v>
       </c>
     </row>
     <row r="323" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A323" t="s">
-        <v>411</v>
+        <v>405</v>
       </c>
       <c r="B323" t="s">
         <v>285</v>
@@ -7311,12 +7320,12 @@
         <v>187</v>
       </c>
       <c r="D323" t="s">
-        <v>412</v>
+        <v>406</v>
       </c>
     </row>
     <row r="324" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A324" t="s">
-        <v>413</v>
+        <v>407</v>
       </c>
       <c r="B324" t="s">
         <v>285</v>
@@ -7325,12 +7334,12 @@
         <v>187</v>
       </c>
       <c r="D324" t="s">
-        <v>414</v>
+        <v>408</v>
       </c>
     </row>
     <row r="325" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A325" t="s">
-        <v>415</v>
+        <v>409</v>
       </c>
       <c r="B325" t="s">
         <v>285</v>
@@ -7339,12 +7348,12 @@
         <v>187</v>
       </c>
       <c r="D325" t="s">
-        <v>416</v>
+        <v>410</v>
       </c>
     </row>
     <row r="326" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A326" t="s">
-        <v>417</v>
+        <v>411</v>
       </c>
       <c r="B326" t="s">
         <v>285</v>
@@ -7353,12 +7362,12 @@
         <v>187</v>
       </c>
       <c r="D326" t="s">
-        <v>418</v>
+        <v>412</v>
       </c>
     </row>
     <row r="327" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
-        <v>419</v>
+        <v>413</v>
       </c>
       <c r="B327" t="s">
         <v>285</v>
@@ -7367,12 +7376,12 @@
         <v>187</v>
       </c>
       <c r="D327" t="s">
-        <v>420</v>
+        <v>414</v>
       </c>
     </row>
     <row r="328" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A328" t="s">
-        <v>421</v>
+        <v>415</v>
       </c>
       <c r="B328" t="s">
         <v>285</v>
@@ -7381,12 +7390,12 @@
         <v>187</v>
       </c>
       <c r="D328" t="s">
-        <v>422</v>
+        <v>416</v>
       </c>
     </row>
     <row r="329" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A329" t="s">
-        <v>423</v>
+        <v>417</v>
       </c>
       <c r="B329" t="s">
         <v>285</v>
@@ -7395,12 +7404,12 @@
         <v>187</v>
       </c>
       <c r="D329" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
     </row>
     <row r="330" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A330" t="s">
-        <v>425</v>
+        <v>419</v>
       </c>
       <c r="B330" t="s">
         <v>285</v>
@@ -7409,12 +7418,12 @@
         <v>187</v>
       </c>
       <c r="D330" t="s">
-        <v>426</v>
+        <v>420</v>
       </c>
     </row>
     <row r="331" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A331" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
       <c r="B331" t="s">
         <v>285</v>
@@ -7423,12 +7432,12 @@
         <v>187</v>
       </c>
       <c r="D331" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
     </row>
     <row r="332" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A332" t="s">
-        <v>429</v>
+        <v>423</v>
       </c>
       <c r="B332" t="s">
         <v>285</v>
@@ -7437,12 +7446,12 @@
         <v>187</v>
       </c>
       <c r="D332" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
     </row>
     <row r="333" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>431</v>
+        <v>425</v>
       </c>
       <c r="B333" t="s">
         <v>285</v>
@@ -7451,12 +7460,12 @@
         <v>187</v>
       </c>
       <c r="D333" t="s">
-        <v>432</v>
+        <v>426</v>
       </c>
     </row>
     <row r="334" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A334" t="s">
-        <v>433</v>
+        <v>427</v>
       </c>
       <c r="B334" t="s">
         <v>285</v>
@@ -7465,82 +7474,82 @@
         <v>187</v>
       </c>
       <c r="D334" t="s">
-        <v>434</v>
+        <v>428</v>
       </c>
     </row>
     <row r="335" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A335" t="s">
-        <v>264</v>
+        <v>429</v>
       </c>
       <c r="B335" t="s">
         <v>285</v>
       </c>
       <c r="C335" t="s">
-        <v>248</v>
+        <v>187</v>
       </c>
       <c r="D335" t="s">
-        <v>265</v>
+        <v>430</v>
       </c>
     </row>
     <row r="336" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A336" t="s">
-        <v>266</v>
+        <v>431</v>
       </c>
       <c r="B336" t="s">
         <v>285</v>
       </c>
       <c r="C336" t="s">
-        <v>248</v>
+        <v>187</v>
       </c>
       <c r="D336" t="s">
-        <v>267</v>
+        <v>432</v>
       </c>
     </row>
     <row r="337" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A337" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="B337" t="s">
         <v>285</v>
       </c>
       <c r="C337" t="s">
-        <v>7</v>
+        <v>187</v>
       </c>
       <c r="D337" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
     </row>
     <row r="338" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A338" t="s">
-        <v>437</v>
+        <v>264</v>
       </c>
       <c r="B338" t="s">
         <v>285</v>
       </c>
       <c r="C338" t="s">
-        <v>7</v>
+        <v>248</v>
       </c>
       <c r="D338" t="s">
-        <v>438</v>
+        <v>265</v>
       </c>
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A339" t="s">
-        <v>439</v>
+        <v>266</v>
       </c>
       <c r="B339" t="s">
         <v>285</v>
       </c>
       <c r="C339" t="s">
-        <v>7</v>
+        <v>248</v>
       </c>
       <c r="D339" t="s">
-        <v>440</v>
+        <v>267</v>
       </c>
     </row>
     <row r="340" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A340" t="s">
-        <v>441</v>
+        <v>435</v>
       </c>
       <c r="B340" t="s">
         <v>285</v>
@@ -7549,12 +7558,12 @@
         <v>7</v>
       </c>
       <c r="D340" t="s">
-        <v>442</v>
+        <v>436</v>
       </c>
     </row>
     <row r="341" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A341" t="s">
-        <v>443</v>
+        <v>437</v>
       </c>
       <c r="B341" t="s">
         <v>285</v>
@@ -7563,12 +7572,12 @@
         <v>7</v>
       </c>
       <c r="D341" t="s">
-        <v>444</v>
+        <v>438</v>
       </c>
     </row>
     <row r="342" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A342" t="s">
-        <v>445</v>
+        <v>439</v>
       </c>
       <c r="B342" t="s">
         <v>285</v>
@@ -7577,12 +7586,12 @@
         <v>7</v>
       </c>
       <c r="D342" t="s">
-        <v>446</v>
+        <v>440</v>
       </c>
     </row>
     <row r="343" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A343" t="s">
-        <v>447</v>
+        <v>441</v>
       </c>
       <c r="B343" t="s">
         <v>285</v>
@@ -7591,12 +7600,12 @@
         <v>7</v>
       </c>
       <c r="D343" t="s">
-        <v>448</v>
+        <v>442</v>
       </c>
     </row>
     <row r="344" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A344" t="s">
-        <v>449</v>
+        <v>443</v>
       </c>
       <c r="B344" t="s">
         <v>285</v>
@@ -7605,12 +7614,12 @@
         <v>7</v>
       </c>
       <c r="D344" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
     </row>
     <row r="345" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A345" t="s">
-        <v>451</v>
+        <v>445</v>
       </c>
       <c r="B345" t="s">
         <v>285</v>
@@ -7619,12 +7628,12 @@
         <v>7</v>
       </c>
       <c r="D345" t="s">
-        <v>452</v>
+        <v>446</v>
       </c>
     </row>
     <row r="346" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A346" t="s">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="B346" t="s">
         <v>285</v>
@@ -7633,12 +7642,12 @@
         <v>7</v>
       </c>
       <c r="D346" t="s">
-        <v>454</v>
+        <v>448</v>
       </c>
     </row>
     <row r="347" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A347" t="s">
-        <v>455</v>
+        <v>449</v>
       </c>
       <c r="B347" t="s">
         <v>285</v>
@@ -7647,12 +7656,12 @@
         <v>7</v>
       </c>
       <c r="D347" t="s">
-        <v>456</v>
+        <v>450</v>
       </c>
     </row>
     <row r="348" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A348" t="s">
-        <v>457</v>
+        <v>451</v>
       </c>
       <c r="B348" t="s">
         <v>285</v>
@@ -7661,25 +7670,67 @@
         <v>7</v>
       </c>
       <c r="D348" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
     </row>
     <row r="349" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A349" t="s">
+        <v>453</v>
+      </c>
+      <c r="B349" t="s">
+        <v>285</v>
+      </c>
+      <c r="C349" t="s">
+        <v>7</v>
+      </c>
+      <c r="D349" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="350" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A350" t="s">
+        <v>455</v>
+      </c>
+      <c r="B350" t="s">
+        <v>285</v>
+      </c>
+      <c r="C350" t="s">
+        <v>7</v>
+      </c>
+      <c r="D350" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="351" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A351" t="s">
+        <v>457</v>
+      </c>
+      <c r="B351" t="s">
+        <v>285</v>
+      </c>
+      <c r="C351" t="s">
+        <v>7</v>
+      </c>
+      <c r="D351" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="352" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A352" t="s">
         <v>459</v>
       </c>
-      <c r="B349" t="s">
-        <v>285</v>
-      </c>
-      <c r="C349" t="s">
-        <v>7</v>
-      </c>
-      <c r="D349" t="s">
+      <c r="B352" t="s">
+        <v>285</v>
+      </c>
+      <c r="C352" t="s">
+        <v>7</v>
+      </c>
+      <c r="D352" t="s">
         <v>460</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F349" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:F352" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>